<commit_message>
Charge email by sends or clicks, not both
Agentic Engage email is metered one way: 1 credit = 1M emails sent OR
1 credit = 20K email clicks. Add a "Charge email by" choice in the HTML
and a matching dropdown in the workbook (D21); only the chosen metric
counts. SMS and Mobile Push still add on top. The Excel export records
the choice.

Co-Authored-By: Treasure Work <291137728+treasure-work@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ai-credit-calculator.xlsx
+++ b/ai-credit-calculator.xlsx
@@ -329,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -506,6 +506,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -803,7 +805,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>Enter monthly volumes in the yellow cells.</t>
         </is>
@@ -873,24 +875,24 @@
       </c>
       <c r="C7" s="64" t="inlineStr">
         <is>
-          <t># of emails sent / mo. (M)</t>
+          <t># of emails sent / mo. (M) — counts if D21 = Emails sent</t>
         </is>
       </c>
       <c r="D7" s="65" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="66">
-        <f>D7/$H$8</f>
+        <f>IF($D$21="Emails sent",D7/$H$8,0)</f>
         <v/>
       </c>
       <c r="F7" s="66">
         <f>E7*12</f>
         <v/>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="0" t="n">
         <v>600</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="0" t="inlineStr">
         <is>
           <t>Conversations</t>
         </is>
@@ -900,26 +902,26 @@
       <c r="B8" s="64" t="inlineStr"/>
       <c r="C8" s="64" t="inlineStr">
         <is>
-          <t># of email clicks / mo. (K)</t>
+          <t># of email clicks / mo. (K) — counts if D21 = Email clicks</t>
         </is>
       </c>
       <c r="D8" s="65" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="66">
-        <f>D8/$H$9</f>
+        <f>IF($D$21="Email clicks",D8/$H$9,0)</f>
         <v/>
       </c>
       <c r="F8" s="66">
         <f>E8*12</f>
         <v/>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>Million Email Messages</t>
+          <t>Million Email Messages (or clicks below — choose one)</t>
         </is>
       </c>
     </row>
@@ -941,12 +943,12 @@
         <f>E9*12</f>
         <v/>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>Thousand Email Clicks</t>
+          <t>Thousand Email Clicks (or sends above — choose one)</t>
         </is>
       </c>
     </row>
@@ -968,10 +970,10 @@
         <f>E10*12</f>
         <v/>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="0" t="inlineStr">
         <is>
           <t>Thousand SMS Messages</t>
         </is>
@@ -999,10 +1001,10 @@
         <f>E11*12</f>
         <v/>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="0" t="inlineStr">
         <is>
           <t>Million Mobile Push Messages</t>
         </is>
@@ -1026,10 +1028,10 @@
         <f>E12*12</f>
         <v/>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="0" t="inlineStr">
         <is>
           <t>Million RT Profiles (incurred monthly)</t>
         </is>
@@ -1057,10 +1059,10 @@
         <f>E13*12</f>
         <v/>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="0" t="inlineStr">
         <is>
           <t>Million Personalization Calls</t>
         </is>
@@ -1084,10 +1086,10 @@
         <f>E14*12</f>
         <v/>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="0" t="inlineStr">
         <is>
           <t>Million Incoming RT Trigger Events</t>
         </is>
@@ -1111,10 +1113,10 @@
         <f>E15*12</f>
         <v/>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="0" t="inlineStr">
         <is>
           <t>Million Outgoing RT Trigger Activations</t>
         </is>
@@ -1142,10 +1144,10 @@
         <f>E16*12</f>
         <v/>
       </c>
-      <c r="H16" t="n">
+      <c r="H16" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="0" t="inlineStr">
         <is>
           <t>Million Predictions - ML Models</t>
         </is>
@@ -1169,10 +1171,10 @@
         <f>E17*12</f>
         <v/>
       </c>
-      <c r="H17" t="n">
+      <c r="H17" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="0" t="inlineStr">
         <is>
           <t>Million Predictions - RFM Model</t>
         </is>
@@ -1206,7 +1208,7 @@
         <f>F18*E19</f>
         <v/>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="0" t="inlineStr">
         <is>
           <t>AI Signals is included with AEP; credits are based on predictions only.</t>
         </is>
@@ -1223,13 +1225,23 @@
         <f>F18+F19</f>
         <v/>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="0" t="inlineStr">
         <is>
           <t>RT Profiles are charged once across RT Personalization and RT Triggers.</t>
         </is>
       </c>
     </row>
     <row r="21">
+      <c r="C21" s="74" t="inlineStr">
+        <is>
+          <t>Email charged by (choose one)</t>
+        </is>
+      </c>
+      <c r="D21" s="75" t="inlineStr">
+        <is>
+          <t>Emails sent</t>
+        </is>
+      </c>
       <c r="E21" s="69" t="n"/>
       <c r="F21" s="69" t="n"/>
     </row>
@@ -1273,9 +1285,12 @@
       <c r="F24" s="69" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"0%,5%,10%"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Emails sent,Email clicks"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>